<commit_message>
Created objects for the electrical subsystem
</commit_message>
<xml_diff>
--- a/5. Bill of Material.xlsx
+++ b/5. Bill of Material.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Engineering Workflow methodology\3. Engineering Design of Each Subsystem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Energy Management system with deep reinforcement learning\Engineering Workflow methodology\Energy Management system with deep reinforcement learning Project started\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98DADD5-BA1F-4505-9E6E-5729F3D67EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2C9CEF-ECE7-48D4-A332-11B3317E2657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{A2B12B88-2F78-4C11-A603-F2E066252FE8}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="63">
   <si>
     <t>D1</t>
   </si>
@@ -169,51 +169,6 @@
     <t>IR sensor x2</t>
   </si>
   <si>
-    <t>Ply wood Board</t>
-  </si>
-  <si>
-    <t>Batton wood</t>
-  </si>
-  <si>
-    <t>Flex wire</t>
-  </si>
-  <si>
-    <t>Jumper Wire</t>
-  </si>
-  <si>
-    <t>Cat 5 Wire</t>
-  </si>
-  <si>
-    <t>Switches</t>
-  </si>
-  <si>
-    <t>Buttons</t>
-  </si>
-  <si>
-    <t>Hot glue</t>
-  </si>
-  <si>
-    <t>Ephostic gum</t>
-  </si>
-  <si>
-    <t>Nails (Different sizes)</t>
-  </si>
-  <si>
-    <t>Screws of Different sizes</t>
-  </si>
-  <si>
-    <t>Brackets</t>
-  </si>
-  <si>
-    <t>Bearings</t>
-  </si>
-  <si>
-    <t>Shaft rods</t>
-  </si>
-  <si>
-    <t>Ceiling board</t>
-  </si>
-  <si>
     <t>Power Adaptor</t>
   </si>
   <si>
@@ -238,10 +193,40 @@
     <t>Others</t>
   </si>
   <si>
-    <t>Logistics</t>
-  </si>
-  <si>
     <t>Materials</t>
+  </si>
+  <si>
+    <t>Solar panel</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>100 W</t>
+  </si>
+  <si>
+    <t>Fuse</t>
+  </si>
+  <si>
+    <t>Schottky Diode</t>
+  </si>
+  <si>
+    <t>XL406 10A Buck Converter</t>
+  </si>
+  <si>
+    <t>Battery (3S 30P) 1.5Ah 3.7V</t>
+  </si>
+  <si>
+    <t>3 Relays</t>
+  </si>
+  <si>
+    <t>12V Fan</t>
+  </si>
+  <si>
+    <t>Ballancer</t>
+  </si>
+  <si>
+    <t>INA226 Sensor</t>
   </si>
 </sst>
 </file>
@@ -979,201 +964,192 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B960F693-FFA2-4FC4-A5DB-361E8DAE6F1F}">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="23.25" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="76.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="59.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="33.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="44.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="2">
-        <v>16000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
+        <v>52</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="2">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="2">
-        <v>5000</v>
-      </c>
-      <c r="C3" s="6">
-        <f>SUM(B1:B32)</f>
-        <v>87000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
+        <v>55</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="6">
+        <f>SUM(C1:C32)</f>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="7"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="2">
-        <v>5000</v>
-      </c>
-      <c r="C4" s="7"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="2">
-        <v>8000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B5" s="4"/>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="2">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="2">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" s="2">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="2">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="2">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="2">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="2">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="2">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" s="2">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B17" s="2">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="4"/>
-      <c r="B18" s="2"/>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B18" s="4"/>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="4"/>
-      <c r="B19" s="2"/>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B19" s="4"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="4"/>
-      <c r="B20" s="2"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B20" s="4"/>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="4"/>
-      <c r="B21" s="2"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B21" s="4"/>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="4"/>
-      <c r="B22" s="2"/>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B22" s="4"/>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="4"/>
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B23" s="4"/>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="4"/>
-      <c r="B24" s="2"/>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B24" s="4"/>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1197,10 +1173,10 @@
         <v>18</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>20</v>
@@ -1211,7 +1187,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="B2" s="4">
         <v>1</v>
@@ -1226,7 +1202,7 @@
     </row>
     <row r="3" spans="1:5" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B3" s="4">
         <v>4</v>
@@ -1245,7 +1221,7 @@
     </row>
     <row r="4" spans="1:5" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B4" s="4">
         <v>1</v>
@@ -1420,7 +1396,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>20</v>
@@ -1431,7 +1407,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="B2" s="2">
         <v>60000</v>
@@ -1439,7 +1415,7 @@
     </row>
     <row r="3" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="B3" s="2">
         <v>40000</v>
@@ -1570,8 +1546,8 @@
     </row>
     <row r="3" spans="1:1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A3" s="6">
-        <f>SUM(Electronics!E3,Miscellenous!C3,Power!E3,Workmanship!C3)</f>
-        <v>410500</v>
+        <f>SUM(Electronics!E3,Miscellenous!D3,Power!E3,Workmanship!C3)</f>
+        <v>353500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bill of material generation
</commit_message>
<xml_diff>
--- a/5. Bill of Material.xlsx
+++ b/5. Bill of Material.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Energy Management system with deep reinforcement learning\Engineering Workflow methodology\Energy Management system with deep reinforcement learning Project started\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2C9CEF-ECE7-48D4-A332-11B3317E2657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D48427-3AC5-465C-8EED-92E2A70ECCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{A2B12B88-2F78-4C11-A603-F2E066252FE8}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="81">
   <si>
     <t>D1</t>
   </si>
@@ -217,16 +217,70 @@
     <t>Battery (3S 30P) 1.5Ah 3.7V</t>
   </si>
   <si>
-    <t>3 Relays</t>
-  </si>
-  <si>
-    <t>12V Fan</t>
-  </si>
-  <si>
     <t>Ballancer</t>
   </si>
   <si>
-    <t>INA226 Sensor</t>
+    <t>BMS</t>
+  </si>
+  <si>
+    <t>CC/CV 5A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LM2596 Buck Converter </t>
+  </si>
+  <si>
+    <t>5 v</t>
+  </si>
+  <si>
+    <t>Relays</t>
+  </si>
+  <si>
+    <t>10A</t>
+  </si>
+  <si>
+    <t>Bulb</t>
+  </si>
+  <si>
+    <t>5v 2A</t>
+  </si>
+  <si>
+    <t>Fan</t>
+  </si>
+  <si>
+    <t>12v 2A</t>
+  </si>
+  <si>
+    <t>USB Buck converter Module</t>
+  </si>
+  <si>
+    <t>5v 3A</t>
+  </si>
+  <si>
+    <t>ESP32</t>
+  </si>
+  <si>
+    <t>3.7v 1.5Ah</t>
+  </si>
+  <si>
+    <t>Overall Cost</t>
+  </si>
+  <si>
+    <t>Technical cost</t>
+  </si>
+  <si>
+    <t>3s 6A</t>
+  </si>
+  <si>
+    <t>3s 10A</t>
+  </si>
+  <si>
+    <t>0-36V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INA226 Current and Voltage Sensor </t>
+  </si>
+  <si>
+    <t>Trainning the Ai Model</t>
   </si>
 </sst>
 </file>
@@ -307,7 +361,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -318,6 +372,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -964,192 +1027,386 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B960F693-FFA2-4FC4-A5DB-361E8DAE6F1F}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="23.25" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="76.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="44.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" customWidth="1"/>
+    <col min="3" max="4" width="33.85546875" style="10" customWidth="1"/>
+    <col min="5" max="5" width="44.7109375" style="10" customWidth="1"/>
+    <col min="6" max="6" width="21.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>51</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="F1" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="9">
+        <v>1</v>
+      </c>
+      <c r="D2" s="9">
         <v>30000</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="E2" s="8">
+        <f>C2*D2</f>
+        <v>30000</v>
+      </c>
+      <c r="F2" s="8">
+        <f>SUM(E2:E145)</f>
+        <v>243000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A3" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="6">
-        <f>SUM(C1:C32)</f>
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="C3" s="9">
+        <v>1</v>
+      </c>
+      <c r="D3" s="9">
+        <v>500</v>
+      </c>
+      <c r="E3" s="8">
+        <f t="shared" ref="E3:E17" si="0">C3*D3</f>
+        <v>500</v>
+      </c>
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="7"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="9">
+        <v>1</v>
+      </c>
+      <c r="D4" s="9">
+        <v>5000</v>
+      </c>
+      <c r="E4" s="8">
+        <f t="shared" si="0"/>
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="9">
+        <v>3</v>
+      </c>
+      <c r="D5" s="9">
+        <v>8000</v>
+      </c>
+      <c r="E5" s="8">
+        <f t="shared" si="0"/>
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" s="9">
+        <v>1</v>
+      </c>
+      <c r="D6" s="9">
+        <v>3000</v>
+      </c>
+      <c r="E6" s="8">
+        <f t="shared" si="0"/>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B8" s="4"/>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="9">
+        <v>90</v>
+      </c>
+      <c r="D7" s="9">
+        <v>650</v>
+      </c>
+      <c r="E7" s="8">
+        <f t="shared" si="0"/>
+        <v>58500</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" s="9">
+        <v>1</v>
+      </c>
+      <c r="D8" s="9">
+        <v>13000</v>
+      </c>
+      <c r="E8" s="8">
+        <f t="shared" si="0"/>
+        <v>13000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="4"/>
-      <c r="C9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B9" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="9">
+        <v>6</v>
+      </c>
+      <c r="D9" s="9">
+        <v>500</v>
+      </c>
+      <c r="E9" s="8">
+        <f t="shared" si="0"/>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="9">
+        <v>4</v>
+      </c>
+      <c r="D10" s="9">
+        <v>1500</v>
+      </c>
+      <c r="E10" s="8">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="4"/>
+        <v>62</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="9">
+        <v>2</v>
+      </c>
+      <c r="D11" s="9">
+        <v>3000</v>
+      </c>
+      <c r="E11" s="8">
+        <f t="shared" si="0"/>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="9">
+        <v>2</v>
+      </c>
+      <c r="D12" s="9"/>
+      <c r="E12" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="9">
+        <v>1</v>
+      </c>
+      <c r="D13" s="9"/>
+      <c r="E13" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="9">
+        <v>3</v>
+      </c>
+      <c r="D14" s="9">
+        <v>3000</v>
+      </c>
+      <c r="E14" s="8">
+        <f t="shared" si="0"/>
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
+        <v>72</v>
+      </c>
       <c r="B15" s="4"/>
-      <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="4"/>
+      <c r="C15" s="9">
+        <v>1</v>
+      </c>
+      <c r="D15" s="9">
+        <v>20000</v>
+      </c>
+      <c r="E15" s="8">
+        <f t="shared" si="0"/>
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="B16" s="4"/>
-      <c r="C16" s="2"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="4"/>
+      <c r="C16" s="9">
+        <v>1</v>
+      </c>
+      <c r="D16" s="9">
+        <v>15000</v>
+      </c>
+      <c r="E16" s="8">
+        <f t="shared" si="0"/>
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="B17" s="4"/>
-      <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C17" s="9">
+        <v>1</v>
+      </c>
+      <c r="D17" s="9">
+        <v>50000</v>
+      </c>
+      <c r="E17" s="8">
+        <f t="shared" si="0"/>
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="4"/>
       <c r="B18" s="4"/>
-      <c r="C18" s="2"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="8"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="4"/>
       <c r="B19" s="4"/>
-      <c r="C19" s="2"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="8"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="4"/>
       <c r="B20" s="4"/>
-      <c r="C20" s="2"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
-      <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="8"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
-      <c r="C22" s="2"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="8"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="4"/>
       <c r="B23" s="4"/>
-      <c r="C23" s="2"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="2"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1545,9 +1802,9 @@
       </c>
     </row>
     <row r="3" spans="1:1" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A3" s="6">
-        <f>SUM(Electronics!E3,Miscellenous!D3,Power!E3,Workmanship!C3)</f>
-        <v>353500</v>
+      <c r="A3" s="6" t="e">
+        <f>SUM(Electronics!E3,Miscellenous!#REF!,Power!E3,Workmanship!C3)</f>
+        <v>#REF!</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bill of material updated
</commit_message>
<xml_diff>
--- a/5. Bill of Material.xlsx
+++ b/5. Bill of Material.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Energy Management system with deep reinforcement learning\Engineering Workflow methodology\Energy Management system with deep reinforcement learning Project started\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D48427-3AC5-465C-8EED-92E2A70ECCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50589091-3BA4-4CF5-94BF-63A8EE567F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{A2B12B88-2F78-4C11-A603-F2E066252FE8}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="84">
   <si>
     <t>D1</t>
   </si>
@@ -281,6 +281,15 @@
   </si>
   <si>
     <t>Trainning the Ai Model</t>
+  </si>
+  <si>
+    <t>Wire 12AWG</t>
+  </si>
+  <si>
+    <t>Wire 14AWG</t>
+  </si>
+  <si>
+    <t>Miscellaneous</t>
   </si>
 </sst>
 </file>
@@ -1308,63 +1317,86 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="9">
         <v>1</v>
       </c>
-      <c r="D16" s="9">
-        <v>15000</v>
-      </c>
+      <c r="D16" s="9"/>
       <c r="E16" s="8">
         <f t="shared" si="0"/>
-        <v>15000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="9">
         <v>1</v>
       </c>
-      <c r="D17" s="9">
-        <v>50000</v>
-      </c>
+      <c r="D17" s="9"/>
       <c r="E17" s="8">
         <f t="shared" si="0"/>
-        <v>50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="4"/>
+      <c r="A18" s="4" t="s">
+        <v>47</v>
+      </c>
       <c r="B18" s="4"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="8"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="4"/>
+      <c r="A19" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="B19" s="4"/>
-      <c r="C19" s="9"/>
+      <c r="C19" s="9">
+        <v>1</v>
+      </c>
       <c r="D19" s="9"/>
-      <c r="E19" s="8"/>
+      <c r="E19" s="8">
+        <f t="shared" ref="E19:E20" si="1">C19*D19</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="4"/>
+      <c r="A20" s="4" t="s">
+        <v>80</v>
+      </c>
       <c r="B20" s="4"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="8"/>
+      <c r="C20" s="9">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9">
+        <v>15000</v>
+      </c>
+      <c r="E20" s="8">
+        <f t="shared" ref="E20:E21" si="2">C20*D20</f>
+        <v>15000</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="4"/>
+      <c r="A21" s="4" t="s">
+        <v>75</v>
+      </c>
       <c r="B21" s="4"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="8"/>
+      <c r="C21" s="9">
+        <v>1</v>
+      </c>
+      <c r="D21" s="9">
+        <v>50000</v>
+      </c>
+      <c r="E21" s="8">
+        <f t="shared" si="2"/>
+        <v>50000</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="4"/>

</xml_diff>